<commit_message>
769 NE 74th: add OlyBond insulation adhesive (3 @ 1080)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp3FWjZDHZyKTZa15Tj1vA
</commit_message>
<xml_diff>
--- a/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev1.xlsx
+++ b/takeoffs/xlsx/2026-10-20_769_NE_74th_TPO_Takeoff_Rev1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="113">
   <si>
     <t xml:space="preserve">769 NE 74th St — TPO Material Takeoff (GAF EverGuard .060, FULLY BONDED) — Rev 1, 10/20/2026</t>
   </si>
@@ -338,6 +338,15 @@
   </si>
   <si>
     <t xml:space="preserve">Supplier cut list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insulation adhesive (ISO to concrete)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OlyBond 500 (per Marc)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marc 10/20: $1,080 each, 3 needed</t>
   </si>
   <si>
     <t xml:space="preserve">Material subtotal</t>
@@ -356,11 +365,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="\$#,##0.00"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -505,7 +515,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -579,6 +589,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1642,36 +1656,66 @@
         <v>105</v>
       </c>
     </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C39" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="19" t="n">
+        <v>1080</v>
+      </c>
+      <c r="H39" s="19" t="n">
+        <f aca="false">E39*G39</f>
+        <v>3240</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G40" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H40" s="14" t="n">
-        <f aca="false">SUM(H22:H38)</f>
-        <v>19667.98</v>
+        <f aca="false">SUM(H22:H39)</f>
+        <v>22907.98</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G41" s="4" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="H41" s="14" t="n">
         <f aca="false">H40*$C$18</f>
-        <v>1376.7586</v>
+        <v>1603.5586</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="G42" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="H42" s="20" t="n">
+      <c r="G42" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="H42" s="21" t="n">
         <f aca="false">H40+H41</f>
-        <v>21044.7386</v>
+        <v>24511.5386</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>